<commit_message>
Actualización del INFORME 1 con datos técnicos, económicos y diagramas Mermaid
</commit_message>
<xml_diff>
--- a/PCB/BOM_TerraSense.xlsx
+++ b/PCB/BOM_TerraSense.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
   <si>
     <t>Componente</t>
   </si>
@@ -43,6 +43,12 @@
     <t>WROOM-32 confirmado por socios; referencia AFEL 8000 IVA incluido, variante de placa por confirmar</t>
   </si>
   <si>
+    <t>Módulo ambiental Bosch BME280 I2C</t>
+  </si>
+  <si>
+    <t>Precio indicado por socio el 2026-09-05: 3500 CLP; interpretado como precio final con IVA 19%, neto 3500/1.19. Crédito IVA sujeto a factura. Temperatura, humedad relativa y presión locales; no BMP280.</t>
+  </si>
+  <si>
     <t>PCB combinada USB-C carga + boost</t>
   </si>
   <si>
@@ -91,10 +97,16 @@
     <t>No incluye ensamblaje final, ya en personal</t>
   </si>
   <si>
-    <t>Carcasa, prensa estopa, fijaciones y sellado</t>
-  </si>
-  <si>
-    <t>Prototipo; no acredita IP67</t>
+    <t>Carcasa impresa en 3D PETG (servicio externo)</t>
+  </si>
+  <si>
+    <t>Presupuesto neto por conjunto: material, máquina, energía y acabado incluidos; geometría y cotización pendientes. Sin compra de impresora ni duplicar MOD.</t>
+  </si>
+  <si>
+    <t>Prensaestopas, fijaciones, juntas y respiradero BME280</t>
+  </si>
+  <si>
+    <t>Presupuesto neto; ventilación protegida para medir aire exterior, sin encapsular el sensor. No acredita IP67.</t>
   </si>
   <si>
     <t>Cableado y conectores internos adicionales</t>
@@ -444,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="58.7109375" customWidth="1"/>
@@ -513,11 +525,11 @@
         <v>1</v>
       </c>
       <c r="C4">
-        <v>900</v>
+        <v>2941.176470588235</v>
       </c>
       <c r="D4">
         <f>B4*C4</f>
-        <v>900</v>
+        <v>2941.176470588235</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -531,11 +543,11 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>4500</v>
+        <v>900</v>
       </c>
       <c r="D5">
         <f>B5*C5</f>
-        <v>4500</v>
+        <v>900</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
@@ -549,11 +561,11 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>900</v>
+        <v>4500</v>
       </c>
       <c r="D6">
         <f>B6*C6</f>
-        <v>900</v>
+        <v>4500</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -567,11 +579,11 @@
         <v>1</v>
       </c>
       <c r="C7">
-        <v>450</v>
+        <v>900</v>
       </c>
       <c r="D7">
         <f>B7*C7</f>
-        <v>450</v>
+        <v>900</v>
       </c>
       <c r="E7" t="s">
         <v>16</v>
@@ -585,11 +597,11 @@
         <v>1</v>
       </c>
       <c r="C8">
-        <v>250</v>
+        <v>450</v>
       </c>
       <c r="D8">
         <f>B8*C8</f>
-        <v>250</v>
+        <v>450</v>
       </c>
       <c r="E8" t="s">
         <v>18</v>
@@ -600,14 +612,14 @@
         <v>19</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C9">
-        <v>40</v>
+        <v>250</v>
       </c>
       <c r="D9">
         <f>B9*C9</f>
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="E9" t="s">
         <v>20</v>
@@ -618,14 +630,14 @@
         <v>21</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10">
-        <v>1200</v>
+        <v>40</v>
       </c>
       <c r="D10">
         <f>B10*C10</f>
-        <v>1200</v>
+        <v>120</v>
       </c>
       <c r="E10" t="s">
         <v>22</v>
@@ -639,11 +651,11 @@
         <v>1</v>
       </c>
       <c r="C11">
-        <v>2500</v>
+        <v>1200</v>
       </c>
       <c r="D11">
         <f>B11*C11</f>
-        <v>2500</v>
+        <v>1200</v>
       </c>
       <c r="E11" t="s">
         <v>24</v>
@@ -657,11 +669,11 @@
         <v>1</v>
       </c>
       <c r="C12">
-        <v>4500</v>
+        <v>2500</v>
       </c>
       <c r="D12">
         <f>B12*C12</f>
-        <v>4500</v>
+        <v>2500</v>
       </c>
       <c r="E12" t="s">
         <v>26</v>
@@ -675,64 +687,100 @@
         <v>1</v>
       </c>
       <c r="C13">
-        <v>700</v>
+        <v>6000</v>
       </c>
       <c r="D13">
         <f>B13*C13</f>
-        <v>700</v>
+        <v>6000</v>
       </c>
       <c r="E13" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D14">
         <f>B14*C14</f>
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15">
-        <v>2500</v>
+        <v>700</v>
       </c>
       <c r="D15">
         <f>B15*C15</f>
-        <v>2500</v>
+        <v>700</v>
       </c>
       <c r="E15" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>2000</v>
       </c>
       <c r="D16">
-        <f>SUM(D2:D15)</f>
-        <v>75242.68907563025</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
+        <f>B16*C16</f>
+        <v>2000</v>
+      </c>
+      <c r="E16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>2500</v>
+      </c>
+      <c r="D17">
+        <f>B17*C17</f>
+        <v>2500</v>
+      </c>
+      <c r="E17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="D18">
+        <f>SUM(D2:D17)</f>
+        <v>81183.8655462185</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>